<commit_message>
Update AI promt using in week 2
</commit_message>
<xml_diff>
--- a/AIAuditlog.xlsx
+++ b/AIAuditlog.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\POW\Learn\FPT University\Kì 5\SWP391\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\POW\Learn\FPT University\Kì 5\SWP391\Github\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DE8AB9C-953C-427E-8372-D219E300716C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CE5F3BD-F2E6-4EC5-9855-0D77CDCA4E1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="35">
   <si>
     <t>DETAILED AI AUDIT LOG</t>
   </si>
@@ -109,6 +109,42 @@
   </si>
   <si>
     <t>https://docs.google.com/document/d/1YMiXCNmYcuZ2i3TXoPEXApXgWf1L_URewV3G6rTk9Kk/edit?tab=t.0</t>
+  </si>
+  <si>
+    <t>Database Design</t>
+  </si>
+  <si>
+    <t>Cần thiết kế database cho hệ thống kết nối, hỗ trợ nông dân bán hàng nông sản, đảm bảo đáp ứng các chức năng thương mại điện tử và quản lý vận chuyển</t>
+  </si>
+  <si>
+    <t>“Design a database schema for a farmer-enterprise agricultural marketplace system”</t>
+  </si>
+  <si>
+    <t>AI đề xuất các bảng chính: Users, Farmers, Enterprises, Products, Orders, OrderDetails, Payments, Reviews, Deliveries, Categories. Quan hệ: User–Role, Product–Category, Order–Payment, Order–Delivery.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: Schema khá đầy đủ nhưng thiếu yếu tố truy xuất nguồn gốc nông sản và kiểm định chất lượng. Contextualization: Hệ thống tại Việt Nam cần hỗ trợ minh bạch nguồn gốc và trạng thái mùa vụ. Creative Synthesis: Bổ sung thêm các bảng Farm, CropSeason, QualityInspection, ShipmentTracking để phù hợp thực tế nông nghiệp. Decision: Chốt 14 bảng chính gồm Users, Farmers, Enterprises, Products, Categories, Orders, OrderDetails, Payments, Reviews, Deliveries, Farm, CropSeason, QualityInspection, ShipmentTracking để vừa đủ triển khai MVP và dễ mở rộng.</t>
+  </si>
+  <si>
+    <t>https://www.geeksforgeeks.org/how-to-design-a-database-for-online-food-ordering-system/</t>
+  </si>
+  <si>
+    <t>UI/UX Design</t>
+  </si>
+  <si>
+    <t>Cần xây dựng flow screen hợp lý cho hệ thống kết nối, hỗ trợ nông dân bán hàng nông sản để tối ưu trải nghiệm người dùng</t>
+  </si>
+  <si>
+    <t>“Suggest user flow and screen flow for a farmer-enterprise agricultural marketplace application”</t>
+  </si>
+  <si>
+    <t>AI gợi ý flow gồm: Splash Screen, Login/Register, Home, Product Listing, Product Detail, Cart, Checkout, Order Tracking, Profile Dashboard, Admin Panel. Có phân luồng riêng cho Nông dân, Doanh nghiệp và Admin.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: Flow cơ bản phù hợp nhưng chưa phản ánh quy trình giao dịch nông sản thực tế như xác nhận chất lượng và theo dõi vận chuyển. Contextualization: Người dùng chính gồm nông dân và doanh nghiệp nên cần giao diện đơn giản, thao tác nhanh trên điện thoại. Creative Synthesis: Bổ sung các màn hình: Đăng sản phẩm nông sản, Kiểm định chất lượng, Theo dõi vận chuyển, Quản lý mùa vụ, Chat thương lượng giá. Decision: Chốt flow gồm 3 nhóm chính: Buyer Flow, Farmer Flow, Admin Flow với khoảng 15–18 screens đủ cho prototype Figma và phát triển hệ thống.</t>
+  </si>
+  <si>
+    <t>https://www.interaction-design.org/literature/topics/user-flow</t>
   </si>
 </sst>
 </file>
@@ -192,7 +228,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -212,6 +248,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -516,7 +561,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -608,7 +653,7 @@
       <c r="A5" s="2">
         <v>2</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="8" t="s">
         <v>10</v>
       </c>
       <c r="C5" s="2" t="s">
@@ -630,25 +675,57 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
-    </row>
-    <row r="7" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
+    <row r="6" spans="1:8" ht="160.80000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="9">
+        <v>3</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="F6" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G6" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="H6" s="10" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="160.19999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="9">
+        <v>4</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="F7" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="G7" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="H7" s="10" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="8" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2"/>
@@ -830,16 +907,6 @@
       <c r="G25" s="2"/>
       <c r="H25" s="2"/>
     </row>
-    <row r="26" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="2"/>
-      <c r="B26" s="2"/>
-      <c r="C26" s="2"/>
-      <c r="D26" s="2"/>
-      <c r="E26" s="2"/>
-      <c r="F26" s="2"/>
-      <c r="G26" s="2"/>
-      <c r="H26" s="2"/>
-    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:H2"/>
@@ -848,6 +915,8 @@
   <hyperlinks>
     <hyperlink ref="H4" r:id="rId1" xr:uid="{B47353D1-F001-4FAE-AEC9-338AA84DE254}"/>
     <hyperlink ref="H5" r:id="rId2" xr:uid="{C8832F51-635B-4C27-9CA1-0A035AEC2E4C}"/>
+    <hyperlink ref="H6" r:id="rId3" xr:uid="{61A19832-41FF-4B5C-801A-B90B68E267DF}"/>
+    <hyperlink ref="H7" r:id="rId4" xr:uid="{E617F11C-B5AB-456F-A443-E628CFAEEE5E}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update AI promt using in week 3
</commit_message>
<xml_diff>
--- a/AIAuditlog.xlsx
+++ b/AIAuditlog.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\POW\Learn\FPT University\Kì 5\SWP391\Github\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CE5F3BD-F2E6-4EC5-9855-0D77CDCA4E1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35AAEB49-7BE0-487C-BFFA-582BA62576CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="46">
   <si>
     <t>DETAILED AI AUDIT LOG</t>
   </si>
@@ -145,6 +145,39 @@
   </si>
   <si>
     <t>https://www.interaction-design.org/literature/topics/user-flow</t>
+  </si>
+  <si>
+    <t>Homepage Design</t>
+  </si>
+  <si>
+    <t>The team needed to design a homepage that introduces the platform's purpose, highlights agricultural products, and encourages users to explore the marketplace.</t>
+  </si>
+  <si>
+    <t>Suggest a homepage structure for an agricultural e-commerce platform connecting farmers and businesses.</t>
+  </si>
+  <si>
+    <t>AI suggested a homepage containing a hero section, featured products, product categories, search functionality, testimonials, and a call-to-action section.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: Evaluated which sections would provide the most value for first-time visitors.Contextualization: Considered that farmers and buyers may have different browsing behaviors.Creative Synthesis: Combined product showcase and search features into the hero section for easier access.Decision: Implemented a homepage with hero banner, featured products, category display, and navigation menu.</t>
+  </si>
+  <si>
+    <t>Authentication System</t>
+  </si>
+  <si>
+    <t>The platform required a secure authentication system to manage different user roles and protect user data.</t>
+  </si>
+  <si>
+    <t>What authentication features should be included in a web platform for farmers, buyers, and administrators?</t>
+  </si>
+  <si>
+    <t>AI recommended registration, login, password reset, email validation, role-based access control, and session management.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: Reviewed which security features were essential for the MVP version. Contextualization: Considered future expansion with multiple user roles. Creative Synthesis: Combined role selection with the registration process. Decision: Implemented Login, Register, and role-based authentication functionality.</t>
+  </si>
+  <si>
+    <t>https://github.com/POW-VN/AgriMarket</t>
   </si>
 </sst>
 </file>
@@ -242,13 +275,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -257,6 +283,13 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -274,6 +307,72 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>26897</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>8965</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>1156447</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>15391</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{43E6C4F8-BF9E-72D8-6E32-56ECE3F8D3D0}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="12658168" y="9332259"/>
+          <a:ext cx="1129550" cy="1467673"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -574,28 +673,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
-      <c r="F1" s="6"/>
-      <c r="G1" s="6"/>
-      <c r="H1" s="6"/>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
     </row>
     <row r="2" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="6"/>
-      <c r="G2" s="6"/>
-      <c r="H2" s="6"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
     </row>
     <row r="3" spans="1:8" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
@@ -653,7 +752,7 @@
       <c r="A5" s="2">
         <v>2</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B5" s="5" t="s">
         <v>10</v>
       </c>
       <c r="C5" s="2" t="s">
@@ -676,76 +775,105 @@
       </c>
     </row>
     <row r="6" spans="1:8" ht="160.80000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="9">
+      <c r="A6" s="6">
         <v>3</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="C6" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="D6" s="9" t="s">
+      <c r="D6" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="E6" s="9" t="s">
+      <c r="E6" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="F6" s="9" t="s">
+      <c r="F6" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="G6" s="9" t="s">
+      <c r="G6" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="H6" s="10" t="s">
+      <c r="H6" s="7" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="160.19999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="9">
+    <row r="7" spans="1:8" ht="158.4" x14ac:dyDescent="0.3">
+      <c r="A7" s="6">
         <v>4</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="B7" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="C7" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="D7" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="E7" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="F7" s="9" t="s">
+      <c r="F7" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="G7" s="9" t="s">
+      <c r="G7" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="H7" s="10" t="s">
+      <c r="H7" s="7" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="2"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
-    </row>
-    <row r="9" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
+    <row r="8" spans="1:8" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="A8" s="2">
+        <v>5</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A9" s="2">
+        <v>6</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="10" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2"/>
@@ -917,7 +1045,9 @@
     <hyperlink ref="H5" r:id="rId2" xr:uid="{C8832F51-635B-4C27-9CA1-0A035AEC2E4C}"/>
     <hyperlink ref="H6" r:id="rId3" xr:uid="{61A19832-41FF-4B5C-801A-B90B68E267DF}"/>
     <hyperlink ref="H7" r:id="rId4" xr:uid="{E617F11C-B5AB-456F-A443-E628CFAEEE5E}"/>
+    <hyperlink ref="H9" r:id="rId5" xr:uid="{C108FBC7-37CE-4D9C-A79E-DE64AF267891}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing r:id="rId6"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update AI promt using in week 4
</commit_message>
<xml_diff>
--- a/AIAuditlog.xlsx
+++ b/AIAuditlog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\POW\Learn\FPT University\Kì 5\SWP391\Github\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35AAEB49-7BE0-487C-BFFA-582BA62576CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2604C280-FE4D-4B36-8DDE-58A483A01358}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="56">
   <si>
     <t>DETAILED AI AUDIT LOG</t>
   </si>
@@ -178,6 +178,36 @@
   </si>
   <si>
     <t>https://github.com/POW-VN/AgriMarket</t>
+  </si>
+  <si>
+    <t>Farmer Dashboard Screens</t>
+  </si>
+  <si>
+    <t>The team needed interfaces that allow farmers to manage products and view their information efficiently.</t>
+  </si>
+  <si>
+    <t>Suggest key screens for a farmer dashboard in an agricultural marketplace platform.</t>
+  </si>
+  <si>
+    <t>AI proposed Product List, Product Details, Profile Management, Order Overview, and Dashboard Summary screens.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: Selected only the most essential screens for the initial release. Contextualization: Focused on features directly related to product management. Creative Synthesis: Simplified navigation to reduce complexity for non-technical users. Decision: Implemented Farmer Dashboard, Product List, and Farmer Profile screens.</t>
+  </si>
+  <si>
+    <t>Add New Product Feature</t>
+  </si>
+  <si>
+    <t>Farmers needed the ability to create and publish agricultural products on the platform.</t>
+  </si>
+  <si>
+    <t>What information should be included in an Add New Product feature for an agricultural marketplace?</t>
+  </si>
+  <si>
+    <t>AI recommended product name, category, description, price, quantity, image upload, and availability status.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: Determined which fields were mandatory and which could be optional. Contextualization: Considered ease of use for farmers entering product information. Creative Synthesis: Added image upload and simplified product status selection. Decision: Implemented Add New Product functionality with product information form and image upload support.</t>
   </si>
 </sst>
 </file>
@@ -875,25 +905,57 @@
         <v>45</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="2"/>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
-    </row>
-    <row r="11" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
-      <c r="G11" s="2"/>
-      <c r="H11" s="2"/>
+    <row r="10" spans="1:8" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A10" s="2">
+        <v>7</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A11" s="2">
+        <v>8</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="12" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2"/>
@@ -1046,8 +1108,10 @@
     <hyperlink ref="H6" r:id="rId3" xr:uid="{61A19832-41FF-4B5C-801A-B90B68E267DF}"/>
     <hyperlink ref="H7" r:id="rId4" xr:uid="{E617F11C-B5AB-456F-A443-E628CFAEEE5E}"/>
     <hyperlink ref="H9" r:id="rId5" xr:uid="{C108FBC7-37CE-4D9C-A79E-DE64AF267891}"/>
+    <hyperlink ref="H10" r:id="rId6" xr:uid="{A3D9E42F-06E1-4E9C-B11F-BE674AE84FBF}"/>
+    <hyperlink ref="H11" r:id="rId7" xr:uid="{7834E4A4-ABD2-4828-A977-1813C7244DF7}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing r:id="rId6"/>
+  <drawing r:id="rId8"/>
 </worksheet>
 </file>
</xml_diff>